<commit_message>
ukończono transport kolejowy towarowy
</commit_message>
<xml_diff>
--- a/data/dane.xlsx
+++ b/data/dane.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Przemek\Documents\moje dokumenty\studia II\praca magisterska\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Przemek\Documents\moje dokumenty\studia II\praca magisterska\praca-magisterska\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{275155E4-532F-435A-9E53-FF42F2733E93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E80078F5-9C41-497B-B3A0-439E657CFE58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{F84DB0BC-A1A6-46E1-A833-3076C380746F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{F84DB0BC-A1A6-46E1-A833-3076C380746F}"/>
   </bookViews>
   <sheets>
     <sheet name="miesięczne" sheetId="1" r:id="rId1"/>
@@ -320,7 +320,34 @@
         </r>
       </text>
     </comment>
-    <comment ref="E18" authorId="0" shapeId="0" xr:uid="{2EEBD5B5-DAC6-4DDE-9395-939E50BF1FE1}">
+    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{CD321A1E-9082-4914-B0B1-65F37C35F973}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+            <charset val="238"/>
+          </rPr>
+          <t>Przemek:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+            <charset val="238"/>
+          </rPr>
+          <t xml:space="preserve">
+PKB w cenach stałych z 2015 roku w mln euro
+Źródło: Eurostat</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E78" authorId="0" shapeId="0" xr:uid="{2EEBD5B5-DAC6-4DDE-9395-939E50BF1FE1}">
       <text>
         <r>
           <rPr>
@@ -777,219 +804,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="28">
   <si>
     <t>data</t>
-  </si>
-  <si>
-    <t>pas_liczba</t>
-  </si>
-  <si>
-    <t>pas_prac_przew</t>
-  </si>
-  <si>
-    <t>pas_prac_eksp</t>
-  </si>
-  <si>
-    <t>tow_masa</t>
-  </si>
-  <si>
-    <t>tow_prac_przew</t>
-  </si>
-  <si>
-    <t>tow_prac_eksp</t>
-  </si>
-  <si>
-    <t>2010-01-01</t>
-  </si>
-  <si>
-    <t>2010-04-01</t>
-  </si>
-  <si>
-    <t>2010-07-01</t>
-  </si>
-  <si>
-    <t>2010-10-01</t>
-  </si>
-  <si>
-    <t>2011-01-01</t>
-  </si>
-  <si>
-    <t>2011-04-01</t>
-  </si>
-  <si>
-    <t>2011-07-01</t>
-  </si>
-  <si>
-    <t>2011-10-01</t>
-  </si>
-  <si>
-    <t>2012-01-01</t>
-  </si>
-  <si>
-    <t>2012-04-01</t>
-  </si>
-  <si>
-    <t>2012-07-01</t>
-  </si>
-  <si>
-    <t>2012-10-01</t>
-  </si>
-  <si>
-    <t>2013-01-01</t>
-  </si>
-  <si>
-    <t>2013-04-01</t>
-  </si>
-  <si>
-    <t>2013-07-01</t>
-  </si>
-  <si>
-    <t>2013-10-01</t>
-  </si>
-  <si>
-    <t>2014-01-01</t>
-  </si>
-  <si>
-    <t>2014-04-01</t>
-  </si>
-  <si>
-    <t>2014-07-01</t>
-  </si>
-  <si>
-    <t>2014-10-01</t>
-  </si>
-  <si>
-    <t>2015-01-01</t>
-  </si>
-  <si>
-    <t>2015-04-01</t>
-  </si>
-  <si>
-    <t>2015-07-01</t>
-  </si>
-  <si>
-    <t>2015-10-01</t>
-  </si>
-  <si>
-    <t>2016-01-01</t>
-  </si>
-  <si>
-    <t>2016-04-01</t>
-  </si>
-  <si>
-    <t>2016-07-01</t>
-  </si>
-  <si>
-    <t>2016-10-01</t>
-  </si>
-  <si>
-    <t>2017-01-01</t>
-  </si>
-  <si>
-    <t>2017-04-01</t>
-  </si>
-  <si>
-    <t>2017-07-01</t>
-  </si>
-  <si>
-    <t>2017-10-01</t>
-  </si>
-  <si>
-    <t>2018-01-01</t>
-  </si>
-  <si>
-    <t>2018-04-01</t>
-  </si>
-  <si>
-    <t>2018-07-01</t>
-  </si>
-  <si>
-    <t>2018-10-01</t>
-  </si>
-  <si>
-    <t>2019-01-01</t>
-  </si>
-  <si>
-    <t>2019-04-01</t>
-  </si>
-  <si>
-    <t>2019-07-01</t>
-  </si>
-  <si>
-    <t>2019-10-01</t>
-  </si>
-  <si>
-    <t>2020-01-01</t>
-  </si>
-  <si>
-    <t>2020-04-01</t>
-  </si>
-  <si>
-    <t>2020-07-01</t>
-  </si>
-  <si>
-    <t>2020-10-01</t>
-  </si>
-  <si>
-    <t>2021-01-01</t>
-  </si>
-  <si>
-    <t>2021-04-01</t>
-  </si>
-  <si>
-    <t>2021-07-01</t>
-  </si>
-  <si>
-    <t>2021-10-01</t>
-  </si>
-  <si>
-    <t>2022-01-01</t>
-  </si>
-  <si>
-    <t>2022-04-01</t>
-  </si>
-  <si>
-    <t>2022-07-01</t>
-  </si>
-  <si>
-    <t>2022-10-01</t>
-  </si>
-  <si>
-    <t>2023-01-01</t>
-  </si>
-  <si>
-    <t>2023-04-01</t>
-  </si>
-  <si>
-    <t>2023-07-01</t>
-  </si>
-  <si>
-    <t>2023-10-01</t>
-  </si>
-  <si>
-    <t>2024-01-01</t>
-  </si>
-  <si>
-    <t>2024-04-01</t>
-  </si>
-  <si>
-    <t>2024-07-01</t>
-  </si>
-  <si>
-    <t>2024-10-01</t>
-  </si>
-  <si>
-    <t>2025-01-01</t>
-  </si>
-  <si>
-    <t>2025-04-01</t>
-  </si>
-  <si>
-    <t>2025-07-01</t>
-  </si>
-  <si>
-    <t>2025-10-01</t>
   </si>
   <si>
     <t>linie kolejowe eksploatowane [km]</t>
@@ -1051,6 +868,27 @@
   <si>
     <t>emisja gazów cieplarnianych w transporcie kolejowym [tys. ton ekwiwalentu CO2]</t>
   </si>
+  <si>
+    <t>tk_pas_liczba</t>
+  </si>
+  <si>
+    <t>tk_pas_prac_przew</t>
+  </si>
+  <si>
+    <t>tk_pas_prac_eksp</t>
+  </si>
+  <si>
+    <t>tk_tow_masa</t>
+  </si>
+  <si>
+    <t>tk_tow_prac_przew</t>
+  </si>
+  <si>
+    <t>tk_tow_prac_eksp</t>
+  </si>
+  <si>
+    <t>pkb</t>
+  </si>
 </sst>
 </file>
 
@@ -1059,7 +897,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1096,6 +934,13 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="238"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="238"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -1473,22 +1318,22 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="F1" t="s">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="G1" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -5363,1107 +5208,2023 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6302A743-B106-4A34-8F5F-755E294EDE50}">
-  <dimension ref="A1:E65"/>
+  <dimension ref="A1:F125"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="5" width="17.85546875" customWidth="1"/>
+    <col min="2" max="6" width="17.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>79</v>
+        <v>9</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>80</v>
+        <v>10</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>81</v>
+        <v>11</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="2">
+        <v>12</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3">
+        <v>34700</v>
+      </c>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2">
+        <v>44.311999999999998</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3">
+        <v>34790</v>
+      </c>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3">
+        <v>45.125999999999998</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3">
+        <v>34881</v>
+      </c>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4">
+        <v>46.387999999999998</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3">
+        <v>34973</v>
+      </c>
+      <c r="B5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5">
+        <v>46.939</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="3">
+        <v>35065</v>
+      </c>
+      <c r="B6" s="6"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+      <c r="F6">
+        <v>47.94</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="3">
+        <v>35156</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7">
+        <v>48.902000000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="3">
+        <v>35247</v>
+      </c>
+      <c r="B8" s="6"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8">
+        <v>49.441000000000003</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="3">
+        <v>35339</v>
+      </c>
+      <c r="B9" s="6"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9">
+        <v>47.74</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="3">
+        <v>35431</v>
+      </c>
+      <c r="B10" s="6"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10">
+        <v>50.686999999999998</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="3">
+        <v>35521</v>
+      </c>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11">
+        <v>51.390999999999998</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="3">
+        <v>35612</v>
+      </c>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12">
+        <v>51.579000000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="3">
+        <v>35704</v>
+      </c>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13">
+        <v>52.47</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="3">
+        <v>35796</v>
+      </c>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14">
+        <v>53.494</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="3">
+        <v>35886</v>
+      </c>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15">
+        <v>53.496000000000002</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="3">
+        <v>35977</v>
+      </c>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16">
+        <v>54.017000000000003</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="3">
+        <v>36069</v>
+      </c>
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+      <c r="F17">
+        <v>54.192999999999998</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="3">
+        <v>36161</v>
+      </c>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="F18">
+        <v>54.624000000000002</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="3">
+        <v>36251</v>
+      </c>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19">
+        <v>55.784999999999997</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="3">
+        <v>36342</v>
+      </c>
+      <c r="B20" s="6"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="6"/>
+      <c r="E20" s="6"/>
+      <c r="F20">
+        <v>56.902999999999999</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="3">
+        <v>36434</v>
+      </c>
+      <c r="B21" s="6"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+      <c r="F21">
+        <v>57.771999999999998</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="3">
+        <v>36526</v>
+      </c>
+      <c r="B22" s="6"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="6"/>
+      <c r="E22" s="6"/>
+      <c r="F22">
+        <v>58.183</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="3">
+        <v>36617</v>
+      </c>
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+      <c r="F23">
+        <v>58.819000000000003</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="3">
+        <v>36708</v>
+      </c>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+      <c r="F24">
+        <v>59.01</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="3">
+        <v>36800</v>
+      </c>
+      <c r="B25" s="6"/>
+      <c r="C25" s="6"/>
+      <c r="D25" s="6"/>
+      <c r="E25" s="6"/>
+      <c r="F25">
+        <v>60.116999999999997</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="3">
+        <v>36892</v>
+      </c>
+      <c r="B26" s="6"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6"/>
+      <c r="F26">
+        <v>59.88</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="3">
+        <v>36982</v>
+      </c>
+      <c r="B27" s="6"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="6"/>
+      <c r="E27" s="6"/>
+      <c r="F27">
+        <v>59.704999999999998</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="3">
+        <v>37073</v>
+      </c>
+      <c r="B28" s="6"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="6"/>
+      <c r="E28" s="6"/>
+      <c r="F28">
+        <v>59.991</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="3">
+        <v>37165</v>
+      </c>
+      <c r="B29" s="6"/>
+      <c r="C29" s="6"/>
+      <c r="D29" s="6"/>
+      <c r="E29" s="6"/>
+      <c r="F29">
+        <v>59.95</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="3">
+        <v>37257</v>
+      </c>
+      <c r="B30" s="6"/>
+      <c r="C30" s="6"/>
+      <c r="D30" s="6"/>
+      <c r="E30" s="6"/>
+      <c r="F30">
+        <v>60.33</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="3">
+        <v>37347</v>
+      </c>
+      <c r="B31" s="6"/>
+      <c r="C31" s="6"/>
+      <c r="D31" s="6"/>
+      <c r="E31" s="6"/>
+      <c r="F31">
+        <v>60.731000000000002</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="3">
+        <v>37438</v>
+      </c>
+      <c r="B32" s="6"/>
+      <c r="C32" s="6"/>
+      <c r="D32" s="6"/>
+      <c r="E32" s="6"/>
+      <c r="F32">
+        <v>61.31</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="3">
+        <v>37530</v>
+      </c>
+      <c r="B33" s="6"/>
+      <c r="C33" s="6"/>
+      <c r="D33" s="6"/>
+      <c r="E33" s="6"/>
+      <c r="F33">
+        <v>61.619</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" s="3">
+        <v>37622</v>
+      </c>
+      <c r="B34" s="6"/>
+      <c r="C34" s="6"/>
+      <c r="D34" s="6"/>
+      <c r="E34" s="6"/>
+      <c r="F34">
+        <v>61.88</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="3">
+        <v>37712</v>
+      </c>
+      <c r="B35" s="6"/>
+      <c r="C35" s="6"/>
+      <c r="D35" s="6"/>
+      <c r="E35" s="6"/>
+      <c r="F35">
+        <v>62.911999999999999</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="3">
+        <v>37803</v>
+      </c>
+      <c r="B36" s="6"/>
+      <c r="C36" s="6"/>
+      <c r="D36" s="6"/>
+      <c r="E36" s="6"/>
+      <c r="F36">
+        <v>63.722999999999999</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="3">
+        <v>37895</v>
+      </c>
+      <c r="B37" s="6"/>
+      <c r="C37" s="6"/>
+      <c r="D37" s="6"/>
+      <c r="E37" s="6"/>
+      <c r="F37">
+        <v>64.221000000000004</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" s="3">
+        <v>37987</v>
+      </c>
+      <c r="B38" s="6"/>
+      <c r="C38" s="6"/>
+      <c r="D38" s="6"/>
+      <c r="E38" s="6"/>
+      <c r="F38">
+        <v>65.739999999999995</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" s="3">
+        <v>38078</v>
+      </c>
+      <c r="B39" s="6"/>
+      <c r="C39" s="6"/>
+      <c r="D39" s="6"/>
+      <c r="E39" s="6"/>
+      <c r="F39">
+        <v>66.287999999999997</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" s="3">
+        <v>38169</v>
+      </c>
+      <c r="B40" s="6"/>
+      <c r="C40" s="6"/>
+      <c r="D40" s="6"/>
+      <c r="E40" s="6"/>
+      <c r="F40">
+        <v>66.253</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" s="3">
+        <v>38261</v>
+      </c>
+      <c r="B41" s="6"/>
+      <c r="C41" s="6"/>
+      <c r="D41" s="6"/>
+      <c r="E41" s="6"/>
+      <c r="F41">
+        <v>66.900000000000006</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" s="3">
+        <v>38353</v>
+      </c>
+      <c r="B42" s="6"/>
+      <c r="C42" s="6"/>
+      <c r="D42" s="6"/>
+      <c r="E42" s="6"/>
+      <c r="F42">
+        <v>67.271000000000001</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" s="3">
+        <v>38443</v>
+      </c>
+      <c r="B43" s="6"/>
+      <c r="C43" s="6"/>
+      <c r="D43" s="6"/>
+      <c r="E43" s="6"/>
+      <c r="F43">
+        <v>67.582999999999998</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" s="3">
+        <v>38534</v>
+      </c>
+      <c r="B44" s="6"/>
+      <c r="C44" s="6"/>
+      <c r="D44" s="6"/>
+      <c r="E44" s="6"/>
+      <c r="F44">
+        <v>68.801000000000002</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" s="3">
+        <v>38626</v>
+      </c>
+      <c r="B45" s="6"/>
+      <c r="C45" s="6"/>
+      <c r="D45" s="6"/>
+      <c r="E45" s="6"/>
+      <c r="F45">
+        <v>70.037999999999997</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" s="3">
+        <v>38718</v>
+      </c>
+      <c r="B46" s="6"/>
+      <c r="C46" s="6"/>
+      <c r="D46" s="6"/>
+      <c r="E46" s="6"/>
+      <c r="F46">
+        <v>71.132999999999996</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" s="3">
+        <v>38808</v>
+      </c>
+      <c r="B47" s="6"/>
+      <c r="C47" s="6"/>
+      <c r="D47" s="6"/>
+      <c r="E47" s="6"/>
+      <c r="F47">
+        <v>72.784999999999997</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" s="3">
+        <v>38899</v>
+      </c>
+      <c r="B48" s="6"/>
+      <c r="C48" s="6"/>
+      <c r="D48" s="6"/>
+      <c r="E48" s="6"/>
+      <c r="F48">
+        <v>73.971999999999994</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" s="3">
+        <v>38991</v>
+      </c>
+      <c r="B49" s="6"/>
+      <c r="C49" s="6"/>
+      <c r="D49" s="6"/>
+      <c r="E49" s="6"/>
+      <c r="F49">
+        <v>72.950999999999993</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" s="3">
+        <v>39083</v>
+      </c>
+      <c r="B50" s="6"/>
+      <c r="C50" s="6"/>
+      <c r="D50" s="6"/>
+      <c r="E50" s="6"/>
+      <c r="F50">
+        <v>75.957999999999998</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" s="3">
+        <v>39173</v>
+      </c>
+      <c r="B51" s="6"/>
+      <c r="C51" s="6"/>
+      <c r="D51" s="6"/>
+      <c r="E51" s="6"/>
+      <c r="F51">
+        <v>76.95</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" s="3">
+        <v>39264</v>
+      </c>
+      <c r="B52" s="6"/>
+      <c r="C52" s="6"/>
+      <c r="D52" s="6"/>
+      <c r="E52" s="6"/>
+      <c r="F52">
+        <v>78.296999999999997</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" s="3">
+        <v>39356</v>
+      </c>
+      <c r="B53" s="6"/>
+      <c r="C53" s="6"/>
+      <c r="D53" s="6"/>
+      <c r="E53" s="6"/>
+      <c r="F53">
+        <v>79.373000000000005</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" s="3">
+        <v>39448</v>
+      </c>
+      <c r="B54" s="6"/>
+      <c r="C54" s="6"/>
+      <c r="D54" s="6"/>
+      <c r="E54" s="6"/>
+      <c r="F54">
+        <v>80.631</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" s="3">
+        <v>39539</v>
+      </c>
+      <c r="B55" s="6"/>
+      <c r="C55" s="6"/>
+      <c r="D55" s="6"/>
+      <c r="E55" s="6"/>
+      <c r="F55">
+        <v>81.072999999999993</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" s="3">
+        <v>39630</v>
+      </c>
+      <c r="B56" s="6"/>
+      <c r="C56" s="6"/>
+      <c r="D56" s="6"/>
+      <c r="E56" s="6"/>
+      <c r="F56">
+        <v>81.043999999999997</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" s="3">
+        <v>39722</v>
+      </c>
+      <c r="B57" s="6"/>
+      <c r="C57" s="6"/>
+      <c r="D57" s="6"/>
+      <c r="E57" s="6"/>
+      <c r="F57">
+        <v>81.186999999999998</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" s="3">
+        <v>39814</v>
+      </c>
+      <c r="B58" s="6"/>
+      <c r="C58" s="6"/>
+      <c r="D58" s="6"/>
+      <c r="E58" s="6"/>
+      <c r="F58">
+        <v>82.147000000000006</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" s="3">
+        <v>39904</v>
+      </c>
+      <c r="B59" s="6"/>
+      <c r="C59" s="6"/>
+      <c r="D59" s="6"/>
+      <c r="E59" s="6"/>
+      <c r="F59">
+        <v>82.332999999999998</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" s="3">
+        <v>39995</v>
+      </c>
+      <c r="B60" s="6"/>
+      <c r="C60" s="6"/>
+      <c r="D60" s="6"/>
+      <c r="E60" s="6"/>
+      <c r="F60">
+        <v>82.962999999999994</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" s="3">
+        <v>40087</v>
+      </c>
+      <c r="B61" s="6"/>
+      <c r="C61" s="6"/>
+      <c r="D61" s="6"/>
+      <c r="E61" s="6"/>
+      <c r="F61">
+        <v>84.385000000000005</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" s="3">
+        <v>40179</v>
+      </c>
+      <c r="B62" s="2">
         <v>56488</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C62" s="2">
         <v>24674</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D62" s="2">
         <v>1035</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E62" s="2">
         <v>339</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="2">
+      <c r="F62">
+        <v>84.08</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" s="3">
+        <v>40269</v>
+      </c>
+      <c r="B63" s="2">
         <v>54867</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C63" s="2">
         <v>29827</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D63" s="2">
         <v>1324</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E63" s="2">
         <v>539</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="2">
+      <c r="F63">
+        <v>85.331999999999994</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" s="3">
+        <v>40360</v>
+      </c>
+      <c r="B64" s="2">
         <v>50274</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C64" s="2">
         <v>28363</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D64" s="2">
         <v>1527</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E64" s="2">
         <v>697</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="2">
+      <c r="F64">
+        <v>86.334000000000003</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" s="3">
+        <v>40452</v>
+      </c>
+      <c r="B65" s="2">
         <v>58463</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C65" s="2">
         <v>55775</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D65" s="2">
         <v>2396</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E65" s="2">
         <v>941</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="2">
+      <c r="F65">
+        <v>87.051000000000002</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" s="3">
+        <v>40544</v>
+      </c>
+      <c r="B66" s="2">
         <v>67610</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C66" s="2">
         <v>11555</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D66" s="2">
         <v>2917</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E66" s="2">
         <v>564</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="2">
+      <c r="F66">
+        <v>88.616</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" s="3">
+        <v>40634</v>
+      </c>
+      <c r="B67" s="2">
         <v>69213</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C67" s="2">
         <v>12256</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D67" s="2">
         <v>3129</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E67" s="2">
         <v>847</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" s="2">
+      <c r="F67">
+        <v>89.736000000000004</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" s="3">
+        <v>40725</v>
+      </c>
+      <c r="B68" s="2">
         <v>63622</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C68" s="2">
         <v>11373</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D68" s="2">
         <v>2562</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E68" s="2">
         <v>830</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="2">
+      <c r="F68">
+        <v>90.786000000000001</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" s="3">
+        <v>40817</v>
+      </c>
+      <c r="B69" s="2">
         <v>74148</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C69" s="2">
         <v>14840</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D69" s="2">
         <v>3160</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E69" s="2">
         <v>1075</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" s="2">
+      <c r="F69">
+        <v>91.626999999999995</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" s="3">
+        <v>40909</v>
+      </c>
+      <c r="B70" s="2">
         <v>77577</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C70" s="2">
         <v>11091</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D70" s="2">
         <v>2711</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E70" s="2">
         <v>720</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" s="2">
+      <c r="F70">
+        <v>91.822999999999993</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" s="3">
+        <v>41000</v>
+      </c>
+      <c r="B71" s="2">
         <v>71236</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C71" s="2">
         <v>10635</v>
       </c>
-      <c r="D11" s="2">
+      <c r="D71" s="2">
         <v>2958</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E71" s="2">
         <v>802</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B12" s="2">
+      <c r="F71">
+        <v>91.619</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" s="3">
+        <v>41091</v>
+      </c>
+      <c r="B72" s="2">
         <v>57697</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C72" s="2">
         <v>9270</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D72" s="2">
         <v>3175</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E72" s="2">
         <v>629</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B13" s="2">
+      <c r="F72">
+        <v>91.664000000000001</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" s="3">
+        <v>41183</v>
+      </c>
+      <c r="B73" s="2">
         <v>66701</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C73" s="2">
         <v>11648</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D73" s="2">
         <v>2947</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E73" s="2">
         <v>786</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B14" s="2">
+      <c r="F73">
+        <v>91.566999999999993</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" s="3">
+        <v>41275</v>
+      </c>
+      <c r="B74" s="2">
         <v>75906</v>
       </c>
-      <c r="C14" s="2">
+      <c r="C74" s="2">
         <v>10506</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D74" s="2">
         <v>2522</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E74" s="2">
         <v>645</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B15" s="2">
+      <c r="F74">
+        <v>91.316000000000003</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" s="3">
+        <v>41365</v>
+      </c>
+      <c r="B75" s="2">
         <v>72085</v>
       </c>
-      <c r="C15" s="2">
+      <c r="C75" s="2">
         <v>11563</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D75" s="2">
         <v>3179</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E75" s="2">
         <v>838</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B16" s="2">
+      <c r="F75">
+        <v>92.007000000000005</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" s="3">
+        <v>41456</v>
+      </c>
+      <c r="B76" s="2">
         <v>65816</v>
       </c>
-      <c r="C16" s="2">
+      <c r="C76" s="2">
         <v>10297</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D76" s="2">
         <v>3297</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E76" s="2">
         <v>691</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B17" s="2">
+      <c r="F76">
+        <v>92.680999999999997</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" s="3">
+        <v>41548</v>
+      </c>
+      <c r="B77" s="2">
         <v>77176</v>
       </c>
-      <c r="C17" s="2">
+      <c r="C77" s="2">
         <v>14493</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D77" s="2">
         <v>5239</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E77" s="2">
         <v>1013</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B18" s="2">
+      <c r="F77">
+        <v>93.198999999999998</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" s="3">
+        <v>41640</v>
+      </c>
+      <c r="B78" s="2">
         <v>52522</v>
       </c>
-      <c r="C18" s="2">
+      <c r="C78" s="2">
         <v>17589</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D78" s="2">
         <v>1286</v>
       </c>
-      <c r="E18" s="4">
+      <c r="E78" s="4">
         <v>18111</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B19" s="2">
+      <c r="F78">
+        <v>94.445999999999998</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" s="3">
+        <v>41730</v>
+      </c>
+      <c r="B79" s="2">
         <v>77795</v>
       </c>
-      <c r="C19" s="2">
+      <c r="C79" s="2">
         <v>12374</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D79" s="2">
         <v>3139</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E79" s="2">
         <v>910</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B20" s="2">
+      <c r="F79">
+        <v>95.516000000000005</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" s="3">
+        <v>41821</v>
+      </c>
+      <c r="B80" s="2">
         <v>69525</v>
       </c>
-      <c r="C20" s="2">
+      <c r="C80" s="2">
         <v>12455</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D80" s="2">
         <v>2977</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E80" s="2">
         <v>856</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B21" s="2">
+      <c r="F80">
+        <v>96.292000000000002</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" s="3">
+        <v>41913</v>
+      </c>
+      <c r="B81" s="2">
         <v>82517</v>
       </c>
-      <c r="C21" s="2">
+      <c r="C81" s="2">
         <v>14316</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D81" s="2">
         <v>3768</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E81" s="2">
         <v>954</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B22" s="2">
+      <c r="F81">
+        <v>97.111999999999995</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" s="3">
+        <v>42005</v>
+      </c>
+      <c r="B82" s="2">
         <v>92108</v>
       </c>
-      <c r="C22" s="2">
+      <c r="C82" s="2">
         <v>12824</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D82" s="2">
         <v>3552</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E82" s="2">
         <v>982</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B23" s="2">
+      <c r="F82">
+        <v>98.7</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" s="3">
+        <v>42095</v>
+      </c>
+      <c r="B83" s="2">
         <v>86412</v>
       </c>
-      <c r="C23" s="2">
+      <c r="C83" s="2">
         <v>13632</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D83" s="2">
         <v>4351</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E83" s="2">
         <v>1073</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B24" s="2">
+      <c r="F83">
+        <v>99.263999999999996</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" s="3">
+        <v>42186</v>
+      </c>
+      <c r="B84" s="2">
         <v>80826</v>
       </c>
-      <c r="C24" s="2">
+      <c r="C84" s="2">
         <v>13782</v>
       </c>
-      <c r="D24" s="2">
+      <c r="D84" s="2">
         <v>3927</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E84" s="2">
         <v>852</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B25" s="2">
+      <c r="F84">
+        <v>100.59099999999999</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" s="3">
+        <v>42278</v>
+      </c>
+      <c r="B85" s="2">
         <v>96991</v>
       </c>
-      <c r="C25" s="2">
+      <c r="C85" s="2">
         <v>17424</v>
       </c>
-      <c r="D25" s="2">
+      <c r="D85" s="2">
         <v>5094</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E85" s="2">
         <v>1317</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B26" s="2">
+      <c r="F85">
+        <v>101.44499999999999</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" s="3">
+        <v>42370</v>
+      </c>
+      <c r="B86" s="2">
         <v>105236</v>
       </c>
-      <c r="C26" s="2">
+      <c r="C86" s="2">
         <v>14992</v>
       </c>
-      <c r="D26" s="2">
+      <c r="D86" s="2">
         <v>5218</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E86" s="2">
         <v>897</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B27" s="2">
+      <c r="F86">
+        <v>101.264</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" s="3">
+        <v>42461</v>
+      </c>
+      <c r="B87" s="2">
         <v>106486</v>
       </c>
-      <c r="C27" s="2">
+      <c r="C87" s="2">
         <v>17134</v>
       </c>
-      <c r="D27" s="2">
+      <c r="D87" s="2">
         <v>5568</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E87" s="2">
         <v>957</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B28" s="2">
+      <c r="F87">
+        <v>102.75700000000001</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" s="3">
+        <v>42552</v>
+      </c>
+      <c r="B88" s="2">
         <v>92850</v>
       </c>
-      <c r="C28" s="2">
+      <c r="C88" s="2">
         <v>15909</v>
       </c>
-      <c r="D28" s="2">
+      <c r="D88" s="2">
         <v>4773</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E88" s="2">
         <v>1140</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B29" s="2">
+      <c r="F88">
+        <v>103.35599999999999</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" s="3">
+        <v>42644</v>
+      </c>
+      <c r="B89" s="2">
         <v>113486</v>
       </c>
-      <c r="C29" s="2">
+      <c r="C89" s="2">
         <v>16607</v>
       </c>
-      <c r="D29" s="2">
+      <c r="D89" s="2">
         <v>5719</v>
       </c>
-      <c r="E29" s="2">
+      <c r="E89" s="2">
         <v>1209</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B30" s="2">
+      <c r="F89">
+        <v>105.355</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" s="3">
+        <v>42736</v>
+      </c>
+      <c r="B90" s="2">
         <v>127098</v>
       </c>
-      <c r="C30" s="2">
+      <c r="C90" s="2">
         <v>15845</v>
       </c>
-      <c r="D30" s="2">
+      <c r="D90" s="2">
         <v>5107</v>
       </c>
-      <c r="E30" s="2">
+      <c r="E90" s="2">
         <v>1153</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B31" s="2">
+      <c r="F90">
+        <v>106.58799999999999</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" s="3">
+        <v>42826</v>
+      </c>
+      <c r="B91" s="2">
         <v>122628</v>
       </c>
-      <c r="C31" s="2">
+      <c r="C91" s="2">
         <v>16673</v>
       </c>
-      <c r="D31" s="2">
+      <c r="D91" s="2">
         <v>5434</v>
       </c>
-      <c r="E31" s="2">
+      <c r="E91" s="2">
         <v>1129</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B32" s="2">
+      <c r="F91">
+        <v>107.63800000000001</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" s="3">
+        <v>42917</v>
+      </c>
+      <c r="B92" s="2">
         <v>109003</v>
       </c>
-      <c r="C32" s="2">
+      <c r="C92" s="2">
         <v>16001</v>
       </c>
-      <c r="D32" s="2">
+      <c r="D92" s="2">
         <v>4825</v>
       </c>
-      <c r="E32" s="2">
+      <c r="E92" s="2">
         <v>1053</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B33" s="2">
+      <c r="F92">
+        <v>109.252</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" s="3">
+        <v>43009</v>
+      </c>
+      <c r="B93" s="2">
         <v>131922</v>
       </c>
-      <c r="C33" s="2">
+      <c r="C93" s="2">
         <v>18260</v>
       </c>
-      <c r="D33" s="2">
+      <c r="D93" s="2">
         <v>5902</v>
       </c>
-      <c r="E33" s="2">
+      <c r="E93" s="2">
         <v>902</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B34" s="2">
+      <c r="F93">
+        <v>110.806</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" s="3">
+        <v>43101</v>
+      </c>
+      <c r="B94" s="2">
         <v>141872</v>
       </c>
-      <c r="C34" s="2">
+      <c r="C94" s="2">
         <v>16848</v>
       </c>
-      <c r="D34" s="2">
+      <c r="D94" s="2">
         <v>5505</v>
       </c>
-      <c r="E34" s="2">
+      <c r="E94" s="2">
         <v>1004</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B35" s="2">
+      <c r="F94">
+        <v>113.001</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" s="3">
+        <v>43191</v>
+      </c>
+      <c r="B95" s="2">
         <v>136499</v>
       </c>
-      <c r="C35" s="2">
+      <c r="C95" s="2">
         <v>19336</v>
       </c>
-      <c r="D35" s="2">
+      <c r="D95" s="2">
         <v>6106</v>
       </c>
-      <c r="E35" s="2">
+      <c r="E95" s="2">
         <v>1313</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B36" s="2">
+      <c r="F95">
+        <v>114.654</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" s="3">
+        <v>43282</v>
+      </c>
+      <c r="B96" s="2">
         <v>132654</v>
       </c>
-      <c r="C36" s="2">
+      <c r="C96" s="2">
         <v>18278</v>
       </c>
-      <c r="D36" s="2">
+      <c r="D96" s="2">
         <v>5321</v>
       </c>
-      <c r="E36" s="2">
+      <c r="E96" s="2">
         <v>1277</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B37" s="2">
+      <c r="F96">
+        <v>116.10299999999999</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" s="3">
+        <v>43374</v>
+      </c>
+      <c r="B97" s="2">
         <v>129371</v>
       </c>
-      <c r="C37" s="2">
+      <c r="C97" s="2">
         <v>22150</v>
       </c>
-      <c r="D37" s="2">
+      <c r="D97" s="2">
         <v>5879</v>
       </c>
-      <c r="E37" s="2">
+      <c r="E97" s="2">
         <v>1253</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="B38" s="2">
+      <c r="F97">
+        <v>117.23699999999999</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" s="3">
+        <v>43466</v>
+      </c>
+      <c r="B98" s="2">
         <v>140998</v>
       </c>
-      <c r="C38" s="2">
+      <c r="C98" s="2">
         <v>18703</v>
       </c>
-      <c r="D38" s="2">
+      <c r="D98" s="2">
         <v>5939</v>
       </c>
-      <c r="E38" s="2">
+      <c r="E98" s="2">
         <v>1219</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="B39" s="2">
+      <c r="F98">
+        <v>118.938</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" s="3">
+        <v>43556</v>
+      </c>
+      <c r="B99" s="2">
         <v>140091</v>
       </c>
-      <c r="C39" s="2">
+      <c r="C99" s="2">
         <v>20726</v>
       </c>
-      <c r="D39" s="2">
+      <c r="D99" s="2">
         <v>6860</v>
       </c>
-      <c r="E39" s="2">
+      <c r="E99" s="2">
         <v>1387</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="B40" s="2">
+      <c r="F99">
+        <v>120.044</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" s="3">
+        <v>43647</v>
+      </c>
+      <c r="B100" s="2">
         <v>133951</v>
       </c>
-      <c r="C40" s="2">
+      <c r="C100" s="2">
         <v>17405</v>
       </c>
-      <c r="D40" s="2">
+      <c r="D100" s="2">
         <v>3852</v>
       </c>
-      <c r="E40" s="2">
+      <c r="E100" s="2">
         <v>480</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B41" s="2">
+      <c r="F100">
+        <v>120.988</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" s="3">
+        <v>43739</v>
+      </c>
+      <c r="B101" s="2">
         <v>146113</v>
       </c>
-      <c r="C41" s="2">
+      <c r="C101" s="2">
         <v>20397</v>
       </c>
-      <c r="D41" s="2">
+      <c r="D101" s="2">
         <v>3908</v>
       </c>
-      <c r="E41" s="2">
+      <c r="E101" s="2">
         <v>512</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="B42" s="2">
+      <c r="F101">
+        <v>121.851</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" s="3">
+        <v>43831</v>
+      </c>
+      <c r="B102" s="2">
         <v>108842</v>
       </c>
-      <c r="C42" s="2">
+      <c r="C102" s="2">
         <v>14564</v>
       </c>
-      <c r="D42" s="2">
+      <c r="D102" s="2">
         <v>3457</v>
       </c>
-      <c r="E42" s="2">
+      <c r="E102" s="2">
         <v>422</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B43" s="2">
+      <c r="F102">
+        <v>122.584</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" s="3">
+        <v>43922</v>
+      </c>
+      <c r="B103" s="2">
         <v>72945</v>
       </c>
-      <c r="C43" s="2">
+      <c r="C103" s="2">
         <v>11937</v>
       </c>
-      <c r="D43" s="2">
+      <c r="D103" s="2">
         <v>2146</v>
       </c>
-      <c r="E43" s="2">
+      <c r="E103" s="2">
         <v>319</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B44" s="2">
+      <c r="F103">
+        <v>111.55500000000001</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" s="3">
+        <v>44013</v>
+      </c>
+      <c r="B104" s="2">
         <v>116184</v>
       </c>
-      <c r="C44" s="2">
+      <c r="C104" s="2">
         <v>16715</v>
       </c>
-      <c r="D44" s="2">
+      <c r="D104" s="2">
         <v>3472</v>
       </c>
-      <c r="E44" s="2">
+      <c r="E104" s="2">
         <v>376</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="B45" s="2">
+      <c r="F104">
+        <v>118.883</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" s="3">
+        <v>44105</v>
+      </c>
+      <c r="B105" s="2">
         <v>134423</v>
       </c>
-      <c r="C45" s="2">
+      <c r="C105" s="2">
         <v>20455</v>
       </c>
-      <c r="D45" s="2">
+      <c r="D105" s="2">
         <v>5392</v>
       </c>
-      <c r="E45" s="2">
+      <c r="E105" s="2">
         <v>482</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B46" s="2">
+      <c r="F105">
+        <v>119.053</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" s="3">
+        <v>44197</v>
+      </c>
+      <c r="B106" s="2">
         <v>118668</v>
       </c>
-      <c r="C46" s="2">
+      <c r="C106" s="2">
         <v>19292</v>
       </c>
-      <c r="D46" s="2">
+      <c r="D106" s="2">
         <v>5604</v>
       </c>
-      <c r="E46" s="2">
+      <c r="E106" s="2">
         <v>331</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A47" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B47" s="2">
+      <c r="F106">
+        <v>121.84399999999999</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" s="3">
+        <v>44287</v>
+      </c>
+      <c r="B107" s="2">
         <v>125995</v>
       </c>
-      <c r="C47" s="2">
+      <c r="C107" s="2">
         <v>21609</v>
       </c>
-      <c r="D47" s="2">
+      <c r="D107" s="2">
         <v>6399</v>
       </c>
-      <c r="E47" s="2">
+      <c r="E107" s="2">
         <v>391</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="B48" s="2">
+      <c r="F107">
+        <v>124.941</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" s="3">
+        <v>44378</v>
+      </c>
+      <c r="B108" s="2">
         <v>106275</v>
       </c>
-      <c r="C48" s="2">
+      <c r="C108" s="2">
         <v>17721</v>
       </c>
-      <c r="D48" s="2">
+      <c r="D108" s="2">
         <v>5149</v>
       </c>
-      <c r="E48" s="2">
+      <c r="E108" s="2">
         <v>415</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A49" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="B49" s="2">
+      <c r="F108">
+        <v>127.51600000000001</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" s="3">
+        <v>44470</v>
+      </c>
+      <c r="B109" s="2">
         <v>99893</v>
       </c>
-      <c r="C49" s="2">
+      <c r="C109" s="2">
         <v>19918</v>
       </c>
-      <c r="D49" s="2">
+      <c r="D109" s="2">
         <v>7092</v>
       </c>
-      <c r="E49" s="2">
+      <c r="E109" s="2">
         <v>304</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B50" s="2">
+      <c r="F109">
+        <v>130.06100000000001</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" s="3">
+        <v>44562</v>
+      </c>
+      <c r="B110" s="2">
         <v>102326</v>
       </c>
-      <c r="C50" s="2">
+      <c r="C110" s="2">
         <v>17132</v>
       </c>
-      <c r="D50" s="2">
+      <c r="D110" s="2">
         <v>5386</v>
       </c>
-      <c r="E50" s="2">
+      <c r="E110" s="2">
         <v>312</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B51" s="2">
+      <c r="F110">
+        <v>134.35300000000001</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" s="3">
+        <v>44652</v>
+      </c>
+      <c r="B111" s="2">
         <v>110838</v>
       </c>
-      <c r="C51" s="2">
+      <c r="C111" s="2">
         <v>16839</v>
       </c>
-      <c r="D51" s="2">
+      <c r="D111" s="2">
         <v>6312</v>
       </c>
-      <c r="E51" s="2">
+      <c r="E111" s="2">
         <v>264</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="B52" s="2">
+      <c r="F111">
+        <v>132.858</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" s="3">
+        <v>44743</v>
+      </c>
+      <c r="B112" s="2">
         <v>104869</v>
       </c>
-      <c r="C52" s="2">
+      <c r="C112" s="2">
         <v>16002</v>
       </c>
-      <c r="D52" s="2">
+      <c r="D112" s="2">
         <v>6095</v>
       </c>
-      <c r="E52" s="2">
+      <c r="E112" s="2">
         <v>199</v>
       </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="B53" s="2">
+      <c r="F112">
+        <v>133.596</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" s="3">
+        <v>44835</v>
+      </c>
+      <c r="B113" s="2">
         <v>103532</v>
       </c>
-      <c r="C53" s="2">
+      <c r="C113" s="2">
         <v>17644</v>
       </c>
-      <c r="D53" s="2">
+      <c r="D113" s="2">
         <v>8209</v>
       </c>
-      <c r="E53" s="2">
+      <c r="E113" s="2">
         <v>290</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B54" s="2">
+      <c r="F113">
+        <v>131.422</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" s="3">
+        <v>44927</v>
+      </c>
+      <c r="B114" s="2">
         <v>123396</v>
       </c>
-      <c r="C54" s="2">
+      <c r="C114" s="2">
         <v>17505</v>
       </c>
-      <c r="D54" s="2">
+      <c r="D114" s="2">
         <v>6408</v>
       </c>
-      <c r="E54" s="2">
+      <c r="E114" s="2">
         <v>262</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A55" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B55" s="2">
+      <c r="F114">
+        <v>132.70500000000001</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" s="3">
+        <v>45017</v>
+      </c>
+      <c r="B115" s="2">
         <v>116307</v>
       </c>
-      <c r="C55" s="2">
+      <c r="C115" s="2">
         <v>17216</v>
       </c>
-      <c r="D55" s="2">
+      <c r="D115" s="2">
         <v>6439</v>
       </c>
-      <c r="E55" s="2">
+      <c r="E115" s="2">
         <v>369</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A56" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="B56" s="2">
+      <c r="F115">
+        <v>131.89099999999999</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" s="3">
+        <v>45108</v>
+      </c>
+      <c r="B116" s="2">
         <v>112282</v>
       </c>
-      <c r="C56" s="2">
+      <c r="C116" s="2">
         <v>17492</v>
       </c>
-      <c r="D56" s="2">
+      <c r="D116" s="2">
         <v>6658</v>
       </c>
-      <c r="E56" s="2">
+      <c r="E116" s="2">
         <v>430</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A57" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="B57" s="2">
+      <c r="F116">
+        <v>134.435</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" s="3">
+        <v>45200</v>
+      </c>
+      <c r="B117" s="2">
         <v>125273</v>
       </c>
-      <c r="C57" s="2">
+      <c r="C117" s="2">
         <v>18669</v>
       </c>
-      <c r="D57" s="2">
+      <c r="D117" s="2">
         <v>6157</v>
       </c>
-      <c r="E57" s="2">
+      <c r="E117" s="2">
         <v>505</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A58" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="B58" s="2">
+      <c r="F117">
+        <v>133.96299999999999</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" s="3">
+        <v>45292</v>
+      </c>
+      <c r="B118" s="2">
         <v>139467</v>
       </c>
-      <c r="C58" s="2">
+      <c r="C118" s="2">
         <v>17645</v>
       </c>
-      <c r="D58" s="2">
+      <c r="D118" s="2">
         <v>5262</v>
       </c>
-      <c r="E58" s="2">
+      <c r="E118" s="2">
         <v>486</v>
       </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A59" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="B59" s="2">
+      <c r="F118">
+        <v>135.15799999999999</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" s="3">
+        <v>45383</v>
+      </c>
+      <c r="B119" s="2">
         <v>139326</v>
       </c>
-      <c r="C59" s="2">
+      <c r="C119" s="2">
         <v>18451</v>
       </c>
-      <c r="D59" s="2">
+      <c r="D119" s="2">
         <v>5649</v>
       </c>
-      <c r="E59" s="2">
+      <c r="E119" s="2">
         <v>580</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A60" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="B60" s="2">
+      <c r="F119">
+        <v>137.20699999999999</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" s="3">
+        <v>45474</v>
+      </c>
+      <c r="B120" s="2">
         <v>122238</v>
       </c>
-      <c r="C60" s="2">
+      <c r="C120" s="2">
         <v>16455</v>
       </c>
-      <c r="D60" s="2">
+      <c r="D120" s="2">
         <v>3477</v>
       </c>
-      <c r="E60" s="2">
+      <c r="E120" s="2">
         <v>435</v>
       </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A61" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="B61" s="2">
+      <c r="F120">
+        <v>137.262</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" s="3">
+        <v>45566</v>
+      </c>
+      <c r="B121" s="2">
         <v>153217</v>
       </c>
-      <c r="C61" s="2">
+      <c r="C121" s="2">
         <v>20240</v>
       </c>
-      <c r="D61" s="2">
+      <c r="D121" s="2">
         <v>4452</v>
       </c>
-      <c r="E61" s="2">
+      <c r="E121" s="2">
         <v>628</v>
       </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A62" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="B62" s="2">
+      <c r="F121">
+        <v>139.13300000000001</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" s="3">
+        <v>45658</v>
+      </c>
+      <c r="B122" s="2">
         <v>142953</v>
       </c>
-      <c r="C62" s="2">
+      <c r="C122" s="2">
         <v>17340</v>
       </c>
-      <c r="D62" s="2">
+      <c r="D122" s="2">
         <v>4568</v>
       </c>
-      <c r="E62" s="2">
+      <c r="E122" s="2">
         <v>531</v>
       </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A63" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="B63" s="2">
+      <c r="F122">
+        <v>140.16499999999999</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" s="3">
+        <v>45748</v>
+      </c>
+      <c r="B123" s="2">
         <v>143976</v>
       </c>
-      <c r="C63" s="2">
+      <c r="C123" s="2">
         <v>18121</v>
       </c>
-      <c r="D63" s="2">
+      <c r="D123" s="2">
         <v>6224</v>
       </c>
-      <c r="E63" s="2">
+      <c r="E123" s="2">
         <v>595</v>
       </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A64" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B64" s="2">
+      <c r="F123">
+        <v>141.363</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" s="3">
+        <v>45839</v>
+      </c>
+      <c r="B124" s="2">
         <v>143250</v>
       </c>
-      <c r="C64" s="2">
+      <c r="C124" s="2">
         <v>17278</v>
       </c>
-      <c r="D64" s="2">
+      <c r="D124" s="2">
         <v>4698</v>
       </c>
-      <c r="E64" s="2">
+      <c r="E124" s="2">
         <v>570</v>
       </c>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A65" s="1" t="s">
-        <v>70</v>
+      <c r="F124">
+        <v>142.68799999999999</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" s="3">
+        <v>45931</v>
+      </c>
+      <c r="F125">
+        <v>144.17400000000001</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
@@ -6482,52 +7243,52 @@
         <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>71</v>
+        <v>1</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>72</v>
+        <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>73</v>
+        <v>3</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>74</v>
+        <v>4</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>75</v>
+        <v>5</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>76</v>
+        <v>6</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>77</v>
+        <v>7</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>78</v>
+        <v>8</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>83</v>
+        <v>13</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>84</v>
+        <v>14</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>85</v>
+        <v>15</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>86</v>
+        <v>16</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>87</v>
+        <v>17</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>88</v>
+        <v>18</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>89</v>
+        <v>19</v>
       </c>
       <c r="Q1" s="5" t="s">
-        <v>90</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
ukończono prace nad transportem kolejowym i drogowym
</commit_message>
<xml_diff>
--- a/data/dane.xlsx
+++ b/data/dane.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Przemek\Documents\moje dokumenty\studia II\praca magisterska\praca-magisterska\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E80078F5-9C41-497B-B3A0-439E657CFE58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CDA09B7-4C93-4FCD-99DD-552E9EF9FBE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{F84DB0BC-A1A6-46E1-A833-3076C380746F}"/>
   </bookViews>
@@ -238,6 +238,7 @@
             <charset val="238"/>
           </rPr>
           <t xml:space="preserve">
+zarejestrowane samochody osobowe [szt.]
 Żródło: GUS</t>
         </r>
       </text>
@@ -264,6 +265,7 @@
             <charset val="238"/>
           </rPr>
           <t xml:space="preserve">
+zarejestrowane samochody ciężarowe [szt.]
 Żródło: GUS</t>
         </r>
       </text>
@@ -290,6 +292,7 @@
             <charset val="238"/>
           </rPr>
           <t xml:space="preserve">
+zarejestrowane ciągniki siodłowe [szt.]
 Żródło: GUS</t>
         </r>
       </text>
@@ -316,6 +319,7 @@
             <charset val="238"/>
           </rPr>
           <t xml:space="preserve">
+zarejestrowane autobusy i trolejbusy [szt.]
 Żródło: GUS</t>
         </r>
       </text>
@@ -343,6 +347,87 @@
           </rPr>
           <t xml:space="preserve">
 PKB w cenach stałych z 2015 roku w mln euro
+Źródło: Eurostat</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0" xr:uid="{9ADBB809-0A2A-431A-B341-8C9CFFADDA41}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+            <charset val="238"/>
+          </rPr>
+          <t>Przemek:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+            <charset val="238"/>
+          </rPr>
+          <t xml:space="preserve">
+masa towarów przewiezionych transportem drogowym [tys. ton]
+Źródło: Eurostat</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{D51ACB95-4A2C-4E66-9977-F7591AD469B4}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+            <charset val="238"/>
+          </rPr>
+          <t>Przemek:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+            <charset val="238"/>
+          </rPr>
+          <t xml:space="preserve">
+praca przewozowa w transporcie drogowym towarowym [mln tkm]
+Źródło: Eurostat</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{F0C3D366-8381-44FA-82DF-028AFC2753E5}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+            <charset val="238"/>
+          </rPr>
+          <t>Przemek:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+            <charset val="238"/>
+          </rPr>
+          <t xml:space="preserve">
+praca eksploatacyjna w transporcie drogowym towarowym [mln pojazdokm]
 Źródło: Eurostat</t>
         </r>
       </text>
@@ -804,7 +889,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="31">
   <si>
     <t>data</t>
   </si>
@@ -831,18 +916,6 @@
   </si>
   <si>
     <t>lokomotywy elektryczne [szt.]</t>
-  </si>
-  <si>
-    <t>zarejestrowane samochody osobowe [szt.]</t>
-  </si>
-  <si>
-    <t>zarejestrowane samochody ciężarowe [szt.]</t>
-  </si>
-  <si>
-    <t>zarejestrowane ciągniki siodłowe [szt.]</t>
-  </si>
-  <si>
-    <t>zarejestrowane autobusy i trolejbusy [szt.]</t>
   </si>
   <si>
     <t>drogi publiczne bez autostrad [km]</t>
@@ -888,6 +961,27 @@
   </si>
   <si>
     <t>pkb</t>
+  </si>
+  <si>
+    <t>td_tow_masa</t>
+  </si>
+  <si>
+    <t>td_tow_prac_przew</t>
+  </si>
+  <si>
+    <t>td_tow_prac_eksp</t>
+  </si>
+  <si>
+    <t>td_poj_sam_os</t>
+  </si>
+  <si>
+    <t>td_poj_sam_ciez</t>
+  </si>
+  <si>
+    <t>td_poj_ciag_siod</t>
+  </si>
+  <si>
+    <t>td_poj_ait</t>
   </si>
 </sst>
 </file>
@@ -1318,22 +1412,22 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="C1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
-      </c>
-      <c r="D1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F1" t="s">
-        <v>25</v>
-      </c>
-      <c r="G1" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -5208,34 +5302,43 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6302A743-B106-4A34-8F5F-755E294EDE50}">
-  <dimension ref="A1:F125"/>
+  <dimension ref="A1:I125"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="6" width="17.85546875" customWidth="1"/>
+    <col min="2" max="9" width="17.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>34700</v>
       </c>
@@ -5247,7 +5350,7 @@
         <v>44.311999999999998</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>34790</v>
       </c>
@@ -5259,7 +5362,7 @@
         <v>45.125999999999998</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>34881</v>
       </c>
@@ -5271,7 +5374,7 @@
         <v>46.387999999999998</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>34973</v>
       </c>
@@ -5283,7 +5386,7 @@
         <v>46.939</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>35065</v>
       </c>
@@ -5295,7 +5398,7 @@
         <v>47.94</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>35156</v>
       </c>
@@ -5307,7 +5410,7 @@
         <v>48.902000000000001</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>35247</v>
       </c>
@@ -5319,7 +5422,7 @@
         <v>49.441000000000003</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>35339</v>
       </c>
@@ -5331,7 +5434,7 @@
         <v>47.74</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>35431</v>
       </c>
@@ -5343,7 +5446,7 @@
         <v>50.686999999999998</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>35521</v>
       </c>
@@ -5355,7 +5458,7 @@
         <v>51.390999999999998</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>35612</v>
       </c>
@@ -5367,7 +5470,7 @@
         <v>51.579000000000001</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>35704</v>
       </c>
@@ -5379,7 +5482,7 @@
         <v>52.47</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>35796</v>
       </c>
@@ -5391,7 +5494,7 @@
         <v>53.494</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>35886</v>
       </c>
@@ -5403,7 +5506,7 @@
         <v>53.496000000000002</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>35977</v>
       </c>
@@ -5607,7 +5710,7 @@
         <v>61.31</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
         <v>37530</v>
       </c>
@@ -5619,7 +5722,7 @@
         <v>61.619</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="3">
         <v>37622</v>
       </c>
@@ -5631,7 +5734,7 @@
         <v>61.88</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
         <v>37712</v>
       </c>
@@ -5643,7 +5746,7 @@
         <v>62.911999999999999</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <v>37803</v>
       </c>
@@ -5655,7 +5758,7 @@
         <v>63.722999999999999</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <v>37895</v>
       </c>
@@ -5667,7 +5770,7 @@
         <v>64.221000000000004</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="3">
         <v>37987</v>
       </c>
@@ -5678,8 +5781,17 @@
       <c r="F38">
         <v>65.739999999999995</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G38">
+        <v>136966</v>
+      </c>
+      <c r="H38">
+        <v>23946</v>
+      </c>
+      <c r="I38">
+        <v>3035</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="3">
         <v>38078</v>
       </c>
@@ -5690,8 +5802,17 @@
       <c r="F39">
         <v>66.287999999999997</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G39">
+        <v>191306</v>
+      </c>
+      <c r="H39">
+        <v>27110</v>
+      </c>
+      <c r="I39">
+        <v>3356</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="3">
         <v>38169</v>
       </c>
@@ -5702,8 +5823,17 @@
       <c r="F40">
         <v>66.253</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G40">
+        <v>214226</v>
+      </c>
+      <c r="H40">
+        <v>26524</v>
+      </c>
+      <c r="I40">
+        <v>3317</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="3">
         <v>38261</v>
       </c>
@@ -5714,8 +5844,17 @@
       <c r="F41">
         <v>66.900000000000006</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G41">
+        <v>189552</v>
+      </c>
+      <c r="H41">
+        <v>25227</v>
+      </c>
+      <c r="I41">
+        <v>3165</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="3">
         <v>38353</v>
       </c>
@@ -5726,8 +5865,17 @@
       <c r="F42">
         <v>67.271000000000001</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G42">
+        <v>137605</v>
+      </c>
+      <c r="H42">
+        <v>24152</v>
+      </c>
+      <c r="I42">
+        <v>2897</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="3">
         <v>38443</v>
       </c>
@@ -5738,8 +5886,17 @@
       <c r="F43">
         <v>67.582999999999998</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G43">
+        <v>211544</v>
+      </c>
+      <c r="H43">
+        <v>27222</v>
+      </c>
+      <c r="I43">
+        <v>3228</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="3">
         <v>38534</v>
       </c>
@@ -5750,8 +5907,17 @@
       <c r="F44">
         <v>68.801000000000002</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G44">
+        <v>272931</v>
+      </c>
+      <c r="H44">
+        <v>32426</v>
+      </c>
+      <c r="I44">
+        <v>3571</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="3">
         <v>38626</v>
       </c>
@@ -5762,8 +5928,17 @@
       <c r="F45">
         <v>70.037999999999997</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G45">
+        <v>241316</v>
+      </c>
+      <c r="H45">
+        <v>28026</v>
+      </c>
+      <c r="I45">
+        <v>3315</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="3">
         <v>38718</v>
       </c>
@@ -5774,8 +5949,17 @@
       <c r="F46">
         <v>71.132999999999996</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G46">
+        <v>152571</v>
+      </c>
+      <c r="H46">
+        <v>28079</v>
+      </c>
+      <c r="I46">
+        <v>3138</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="3">
         <v>38808</v>
       </c>
@@ -5786,8 +5970,17 @@
       <c r="F47">
         <v>72.784999999999997</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G47">
+        <v>227915</v>
+      </c>
+      <c r="H47">
+        <v>32888</v>
+      </c>
+      <c r="I47">
+        <v>3572</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="3">
         <v>38899</v>
       </c>
@@ -5798,8 +5991,17 @@
       <c r="F48">
         <v>73.971999999999994</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G48">
+        <v>265433</v>
+      </c>
+      <c r="H48">
+        <v>33048</v>
+      </c>
+      <c r="I48">
+        <v>3764</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="3">
         <v>38991</v>
       </c>
@@ -5810,8 +6012,17 @@
       <c r="F49">
         <v>72.950999999999993</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G49">
+        <v>251496</v>
+      </c>
+      <c r="H49">
+        <v>34300</v>
+      </c>
+      <c r="I49">
+        <v>3803</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="3">
         <v>39083</v>
       </c>
@@ -5822,8 +6033,17 @@
       <c r="F50">
         <v>75.957999999999998</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G50">
+        <v>210232</v>
+      </c>
+      <c r="H50">
+        <v>35982</v>
+      </c>
+      <c r="I50">
+        <v>3753</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" s="3">
         <v>39173</v>
       </c>
@@ -5834,8 +6054,17 @@
       <c r="F51">
         <v>76.95</v>
       </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G51">
+        <v>259801</v>
+      </c>
+      <c r="H51">
+        <v>37930</v>
+      </c>
+      <c r="I51">
+        <v>4004</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="3">
         <v>39264</v>
       </c>
@@ -5846,8 +6075,17 @@
       <c r="F52">
         <v>78.296999999999997</v>
       </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G52">
+        <v>257823</v>
+      </c>
+      <c r="H52">
+        <v>38305</v>
+      </c>
+      <c r="I52">
+        <v>4045</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" s="3">
         <v>39356</v>
       </c>
@@ -5858,8 +6096,17 @@
       <c r="F53">
         <v>79.373000000000005</v>
       </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G53">
+        <v>256381</v>
+      </c>
+      <c r="H53">
+        <v>38663</v>
+      </c>
+      <c r="I53">
+        <v>4102</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" s="3">
         <v>39448</v>
       </c>
@@ -5870,8 +6117,17 @@
       <c r="F54">
         <v>80.631</v>
       </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G54">
+        <v>248087</v>
+      </c>
+      <c r="H54">
+        <v>41390</v>
+      </c>
+      <c r="I54">
+        <v>4185</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" s="3">
         <v>39539</v>
       </c>
@@ -5882,8 +6138,17 @@
       <c r="F55">
         <v>81.072999999999993</v>
       </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G55">
+        <v>275484</v>
+      </c>
+      <c r="H55">
+        <v>44034</v>
+      </c>
+      <c r="I55">
+        <v>4469</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="3">
         <v>39630</v>
       </c>
@@ -5894,8 +6159,17 @@
       <c r="F56">
         <v>81.043999999999997</v>
       </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G56">
+        <v>312901</v>
+      </c>
+      <c r="H56">
+        <v>42254</v>
+      </c>
+      <c r="I56">
+        <v>4370</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" s="3">
         <v>39722</v>
       </c>
@@ -5906,8 +6180,17 @@
       <c r="F57">
         <v>81.186999999999998</v>
       </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G57">
+        <v>256934</v>
+      </c>
+      <c r="H57">
+        <v>37252</v>
+      </c>
+      <c r="I57">
+        <v>3877</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="3">
         <v>39814</v>
       </c>
@@ -5918,8 +6201,17 @@
       <c r="F58">
         <v>82.147000000000006</v>
       </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G58">
+        <v>213214</v>
+      </c>
+      <c r="H58">
+        <v>42755</v>
+      </c>
+      <c r="I58">
+        <v>4323</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" s="3">
         <v>39904</v>
       </c>
@@ -5930,8 +6222,17 @@
       <c r="F59">
         <v>82.332999999999998</v>
       </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G59">
+        <v>303790</v>
+      </c>
+      <c r="H59">
+        <v>45400</v>
+      </c>
+      <c r="I59">
+        <v>4594</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" s="3">
         <v>39995</v>
       </c>
@@ -5942,8 +6243,17 @@
       <c r="F60">
         <v>82.962999999999994</v>
       </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G60">
+        <v>360530</v>
+      </c>
+      <c r="H60">
+        <v>48087</v>
+      </c>
+      <c r="I60">
+        <v>4810</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" s="3">
         <v>40087</v>
       </c>
@@ -5954,8 +6264,17 @@
       <c r="F61">
         <v>84.385000000000005</v>
       </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G61">
+        <v>292944</v>
+      </c>
+      <c r="H61">
+        <v>44500</v>
+      </c>
+      <c r="I61">
+        <v>4372</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" s="3">
         <v>40179</v>
       </c>
@@ -5974,8 +6293,17 @@
       <c r="F62">
         <v>84.08</v>
       </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G62">
+        <v>220124</v>
+      </c>
+      <c r="H62">
+        <v>45790</v>
+      </c>
+      <c r="I62">
+        <v>4327</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" s="3">
         <v>40269</v>
       </c>
@@ -5994,8 +6322,17 @@
       <c r="F63">
         <v>85.331999999999994</v>
       </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G63">
+        <v>334718</v>
+      </c>
+      <c r="H63">
+        <v>51590</v>
+      </c>
+      <c r="I63">
+        <v>4935</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" s="3">
         <v>40360</v>
       </c>
@@ -6014,8 +6351,17 @@
       <c r="F64">
         <v>86.334000000000003</v>
       </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G64">
+        <v>362775</v>
+      </c>
+      <c r="H64">
+        <v>55201</v>
+      </c>
+      <c r="I64">
+        <v>5259</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" s="3">
         <v>40452</v>
       </c>
@@ -6034,8 +6380,17 @@
       <c r="F65">
         <v>87.051000000000002</v>
       </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G65">
+        <v>298466</v>
+      </c>
+      <c r="H65">
+        <v>49727</v>
+      </c>
+      <c r="I65">
+        <v>4777</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" s="3">
         <v>40544</v>
       </c>
@@ -6054,8 +6409,17 @@
       <c r="F66">
         <v>88.616</v>
       </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G66">
+        <v>252367</v>
+      </c>
+      <c r="H66">
+        <v>50581</v>
+      </c>
+      <c r="I66">
+        <v>4664</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" s="3">
         <v>40634</v>
       </c>
@@ -6074,8 +6438,17 @@
       <c r="F67">
         <v>89.736000000000004</v>
       </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G67">
+        <v>355523</v>
+      </c>
+      <c r="H67">
+        <v>52863</v>
+      </c>
+      <c r="I67">
+        <v>4986</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" s="3">
         <v>40725</v>
       </c>
@@ -6094,8 +6467,17 @@
       <c r="F68">
         <v>90.786000000000001</v>
       </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G68">
+        <v>367751</v>
+      </c>
+      <c r="H68">
+        <v>51794</v>
+      </c>
+      <c r="I68">
+        <v>5016</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" s="3">
         <v>40817</v>
       </c>
@@ -6114,8 +6496,17 @@
       <c r="F69">
         <v>91.626999999999995</v>
       </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G69">
+        <v>346596</v>
+      </c>
+      <c r="H69">
+        <v>52412</v>
+      </c>
+      <c r="I69">
+        <v>4973</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" s="3">
         <v>40909</v>
       </c>
@@ -6134,8 +6525,17 @@
       <c r="F70">
         <v>91.822999999999993</v>
       </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G70">
+        <v>250038</v>
+      </c>
+      <c r="H70">
+        <v>53061</v>
+      </c>
+      <c r="I70">
+        <v>4773</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" s="3">
         <v>41000</v>
       </c>
@@ -6154,8 +6554,17 @@
       <c r="F71">
         <v>91.619</v>
       </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G71">
+        <v>327581</v>
+      </c>
+      <c r="H71">
+        <v>57147</v>
+      </c>
+      <c r="I71">
+        <v>5313</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" s="3">
         <v>41091</v>
       </c>
@@ -6174,8 +6583,17 @@
       <c r="F72">
         <v>91.664000000000001</v>
       </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G72">
+        <v>369052</v>
+      </c>
+      <c r="H72">
+        <v>57652</v>
+      </c>
+      <c r="I72">
+        <v>5427</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" s="3">
         <v>41183</v>
       </c>
@@ -6194,8 +6612,17 @@
       <c r="F73">
         <v>91.566999999999993</v>
       </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G73">
+        <v>298382</v>
+      </c>
+      <c r="H73">
+        <v>54472</v>
+      </c>
+      <c r="I73">
+        <v>4967</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" s="3">
         <v>41275</v>
       </c>
@@ -6214,8 +6641,17 @@
       <c r="F74">
         <v>91.316000000000003</v>
       </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G74">
+        <v>240109</v>
+      </c>
+      <c r="H74">
+        <v>57036</v>
+      </c>
+      <c r="I74">
+        <v>5107</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" s="3">
         <v>41365</v>
       </c>
@@ -6234,8 +6670,17 @@
       <c r="F75">
         <v>92.007000000000005</v>
       </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G75">
+        <v>362379</v>
+      </c>
+      <c r="H75">
+        <v>65340</v>
+      </c>
+      <c r="I75">
+        <v>6020</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" s="3">
         <v>41456</v>
       </c>
@@ -6254,8 +6699,17 @@
       <c r="F76">
         <v>92.680999999999997</v>
       </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G76">
+        <v>372003</v>
+      </c>
+      <c r="H76">
+        <v>64602</v>
+      </c>
+      <c r="I76">
+        <v>5911</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" s="3">
         <v>41548</v>
       </c>
@@ -6274,8 +6728,17 @@
       <c r="F77">
         <v>93.198999999999998</v>
       </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G77">
+        <v>326118</v>
+      </c>
+      <c r="H77">
+        <v>60616</v>
+      </c>
+      <c r="I77">
+        <v>5507</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" s="3">
         <v>41640</v>
       </c>
@@ -6294,8 +6757,17 @@
       <c r="F78">
         <v>94.445999999999998</v>
       </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G78">
+        <v>261393</v>
+      </c>
+      <c r="H78">
+        <v>61362</v>
+      </c>
+      <c r="I78">
+        <v>5502</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" s="3">
         <v>41730</v>
       </c>
@@ -6314,8 +6786,17 @@
       <c r="F79">
         <v>95.516000000000005</v>
       </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G79">
+        <v>365960</v>
+      </c>
+      <c r="H79">
+        <v>62808</v>
+      </c>
+      <c r="I79">
+        <v>5714</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" s="3">
         <v>41821</v>
       </c>
@@ -6334,8 +6815,17 @@
       <c r="F80">
         <v>96.292000000000002</v>
       </c>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G80">
+        <v>365997</v>
+      </c>
+      <c r="H80">
+        <v>63343</v>
+      </c>
+      <c r="I80">
+        <v>5694</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81" s="3">
         <v>41913</v>
       </c>
@@ -6354,8 +6844,17 @@
       <c r="F81">
         <v>97.111999999999995</v>
       </c>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G81">
+        <v>307033</v>
+      </c>
+      <c r="H81">
+        <v>63417</v>
+      </c>
+      <c r="I81">
+        <v>5648</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" s="3">
         <v>42005</v>
       </c>
@@ -6374,8 +6873,17 @@
       <c r="F82">
         <v>98.7</v>
       </c>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G82">
+        <v>261787</v>
+      </c>
+      <c r="H82">
+        <v>63257</v>
+      </c>
+      <c r="I82">
+        <v>5836</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" s="3">
         <v>42095</v>
       </c>
@@ -6394,8 +6902,17 @@
       <c r="F83">
         <v>99.263999999999996</v>
       </c>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G83">
+        <v>341508</v>
+      </c>
+      <c r="H83">
+        <v>67679</v>
+      </c>
+      <c r="I83">
+        <v>6202</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84" s="3">
         <v>42186</v>
       </c>
@@ -6414,8 +6931,17 @@
       <c r="F84">
         <v>100.59099999999999</v>
       </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G84">
+        <v>345722</v>
+      </c>
+      <c r="H84">
+        <v>65129</v>
+      </c>
+      <c r="I84">
+        <v>5899</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" s="3">
         <v>42278</v>
       </c>
@@ -6434,8 +6960,17 @@
       <c r="F85">
         <v>101.44499999999999</v>
       </c>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G85">
+        <v>315943</v>
+      </c>
+      <c r="H85">
+        <v>64647</v>
+      </c>
+      <c r="I85">
+        <v>5819</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" s="3">
         <v>42370</v>
       </c>
@@ -6454,8 +6989,17 @@
       <c r="F86">
         <v>101.264</v>
       </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G86">
+        <v>260887</v>
+      </c>
+      <c r="H86">
+        <v>71195</v>
+      </c>
+      <c r="I86">
+        <v>6355</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" s="3">
         <v>42461</v>
       </c>
@@ -6474,8 +7018,17 @@
       <c r="F87">
         <v>102.75700000000001</v>
       </c>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G87">
+        <v>343628</v>
+      </c>
+      <c r="H87">
+        <v>77300</v>
+      </c>
+      <c r="I87">
+        <v>6889</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" s="3">
         <v>42552</v>
       </c>
@@ -6494,8 +7047,17 @@
       <c r="F88">
         <v>103.35599999999999</v>
       </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G88">
+        <v>366574</v>
+      </c>
+      <c r="H88">
+        <v>71533</v>
+      </c>
+      <c r="I88">
+        <v>6462</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" s="3">
         <v>42644</v>
       </c>
@@ -6514,8 +7076,17 @@
       <c r="F89">
         <v>105.355</v>
       </c>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G89">
+        <v>342568</v>
+      </c>
+      <c r="H89">
+        <v>70721</v>
+      </c>
+      <c r="I89">
+        <v>6235</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" s="3">
         <v>42736</v>
       </c>
@@ -6534,8 +7105,17 @@
       <c r="F90">
         <v>106.58799999999999</v>
       </c>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G90">
+        <v>295401</v>
+      </c>
+      <c r="H90">
+        <v>76809</v>
+      </c>
+      <c r="I90">
+        <v>6580</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" s="3">
         <v>42826</v>
       </c>
@@ -6554,8 +7134,17 @@
       <c r="F91">
         <v>107.63800000000001</v>
       </c>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G91">
+        <v>398627</v>
+      </c>
+      <c r="H91">
+        <v>84916</v>
+      </c>
+      <c r="I91">
+        <v>7324</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" s="3">
         <v>42917</v>
       </c>
@@ -6574,8 +7163,17 @@
       <c r="F92">
         <v>109.252</v>
       </c>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G92">
+        <v>415532</v>
+      </c>
+      <c r="H92">
+        <v>86055</v>
+      </c>
+      <c r="I92">
+        <v>7464</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93" s="3">
         <v>43009</v>
       </c>
@@ -6594,8 +7192,17 @@
       <c r="F93">
         <v>110.806</v>
       </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G93">
+        <v>392251</v>
+      </c>
+      <c r="H93">
+        <v>87440</v>
+      </c>
+      <c r="I93">
+        <v>7600</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94" s="3">
         <v>43101</v>
       </c>
@@ -6614,8 +7221,17 @@
       <c r="F94">
         <v>113.001</v>
       </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G94">
+        <v>291009</v>
+      </c>
+      <c r="H94">
+        <v>77946</v>
+      </c>
+      <c r="I94">
+        <v>6849</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95" s="3">
         <v>43191</v>
       </c>
@@ -6634,8 +7250,17 @@
       <c r="F95">
         <v>114.654</v>
       </c>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G95">
+        <v>364897</v>
+      </c>
+      <c r="H95">
+        <v>83132</v>
+      </c>
+      <c r="I95">
+        <v>7211</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A96" s="3">
         <v>43282</v>
       </c>
@@ -6654,8 +7279,17 @@
       <c r="F96">
         <v>116.10299999999999</v>
       </c>
-    </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G96">
+        <v>394544</v>
+      </c>
+      <c r="H96">
+        <v>77624</v>
+      </c>
+      <c r="I96">
+        <v>6733</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97" s="3">
         <v>43374</v>
       </c>
@@ -6674,8 +7308,17 @@
       <c r="F97">
         <v>117.23699999999999</v>
       </c>
-    </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G97">
+        <v>339733</v>
+      </c>
+      <c r="H97">
+        <v>77172</v>
+      </c>
+      <c r="I97">
+        <v>6661</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" s="3">
         <v>43466</v>
       </c>
@@ -6694,8 +7337,17 @@
       <c r="F98">
         <v>118.938</v>
       </c>
-    </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G98">
+        <v>335464</v>
+      </c>
+      <c r="H98">
+        <v>85395</v>
+      </c>
+      <c r="I98">
+        <v>7238</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" s="3">
         <v>43556</v>
       </c>
@@ -6714,8 +7366,17 @@
       <c r="F99">
         <v>120.044</v>
       </c>
-    </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G99">
+        <v>385589</v>
+      </c>
+      <c r="H99">
+        <v>86666</v>
+      </c>
+      <c r="I99">
+        <v>7375</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" s="3">
         <v>43647</v>
       </c>
@@ -6734,8 +7395,17 @@
       <c r="F100">
         <v>120.988</v>
       </c>
-    </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G100">
+        <v>385773</v>
+      </c>
+      <c r="H100">
+        <v>90867</v>
+      </c>
+      <c r="I100">
+        <v>7400</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" s="3">
         <v>43739</v>
       </c>
@@ -6754,8 +7424,17 @@
       <c r="F101">
         <v>121.851</v>
       </c>
-    </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G101">
+        <v>399625</v>
+      </c>
+      <c r="H101">
+        <v>86026</v>
+      </c>
+      <c r="I101">
+        <v>7422</v>
+      </c>
+    </row>
+    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A102" s="3">
         <v>43831</v>
       </c>
@@ -6774,8 +7453,17 @@
       <c r="F102">
         <v>122.584</v>
       </c>
-    </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G102">
+        <v>360608</v>
+      </c>
+      <c r="H102">
+        <v>90262</v>
+      </c>
+      <c r="I102">
+        <v>7616</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A103" s="3">
         <v>43922</v>
       </c>
@@ -6794,8 +7482,17 @@
       <c r="F103">
         <v>111.55500000000001</v>
       </c>
-    </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G103">
+        <v>348505</v>
+      </c>
+      <c r="H103">
+        <v>79863</v>
+      </c>
+      <c r="I103">
+        <v>6945</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A104" s="3">
         <v>44013</v>
       </c>
@@ -6814,8 +7511,17 @@
       <c r="F104">
         <v>118.883</v>
       </c>
-    </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G104">
+        <v>403621</v>
+      </c>
+      <c r="H104">
+        <v>96014</v>
+      </c>
+      <c r="I104">
+        <v>8199</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A105" s="3">
         <v>44105</v>
       </c>
@@ -6834,8 +7540,17 @@
       <c r="F105">
         <v>119.053</v>
       </c>
-    </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G105">
+        <v>387370</v>
+      </c>
+      <c r="H105">
+        <v>88788</v>
+      </c>
+      <c r="I105">
+        <v>7495</v>
+      </c>
+    </row>
+    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A106" s="3">
         <v>44197</v>
       </c>
@@ -6854,8 +7569,17 @@
       <c r="F106">
         <v>121.84399999999999</v>
       </c>
-    </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G106">
+        <v>351425</v>
+      </c>
+      <c r="H106">
+        <v>97073</v>
+      </c>
+      <c r="I106">
+        <v>8140</v>
+      </c>
+    </row>
+    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A107" s="3">
         <v>44287</v>
       </c>
@@ -6874,8 +7598,17 @@
       <c r="F107">
         <v>124.941</v>
       </c>
-    </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G107">
+        <v>409516</v>
+      </c>
+      <c r="H107">
+        <v>96844</v>
+      </c>
+      <c r="I107">
+        <v>8200</v>
+      </c>
+    </row>
+    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A108" s="3">
         <v>44378</v>
       </c>
@@ -6894,8 +7627,17 @@
       <c r="F108">
         <v>127.51600000000001</v>
       </c>
-    </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G108">
+        <v>400901</v>
+      </c>
+      <c r="H108">
+        <v>93380</v>
+      </c>
+      <c r="I108">
+        <v>7946</v>
+      </c>
+    </row>
+    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A109" s="3">
         <v>44470</v>
       </c>
@@ -6914,8 +7656,17 @@
       <c r="F109">
         <v>130.06100000000001</v>
       </c>
-    </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G109">
+        <v>418675</v>
+      </c>
+      <c r="H109">
+        <v>92523</v>
+      </c>
+      <c r="I109">
+        <v>7763</v>
+      </c>
+    </row>
+    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A110" s="3">
         <v>44562</v>
       </c>
@@ -6934,8 +7685,17 @@
       <c r="F110">
         <v>134.35300000000001</v>
       </c>
-    </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G110">
+        <v>392552</v>
+      </c>
+      <c r="H110">
+        <v>104939</v>
+      </c>
+      <c r="I110">
+        <v>8667</v>
+      </c>
+    </row>
+    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A111" s="3">
         <v>44652</v>
       </c>
@@ -6954,8 +7714,17 @@
       <c r="F111">
         <v>132.858</v>
       </c>
-    </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G111">
+        <v>403304</v>
+      </c>
+      <c r="H111">
+        <v>96456</v>
+      </c>
+      <c r="I111">
+        <v>8023</v>
+      </c>
+    </row>
+    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A112" s="3">
         <v>44743</v>
       </c>
@@ -6974,8 +7743,17 @@
       <c r="F112">
         <v>133.596</v>
       </c>
-    </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G112">
+        <v>439169</v>
+      </c>
+      <c r="H112">
+        <v>95629</v>
+      </c>
+      <c r="I112">
+        <v>7982</v>
+      </c>
+    </row>
+    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A113" s="3">
         <v>44835</v>
       </c>
@@ -6994,8 +7772,17 @@
       <c r="F113">
         <v>131.422</v>
       </c>
-    </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G113">
+        <v>364488</v>
+      </c>
+      <c r="H113">
+        <v>88064</v>
+      </c>
+      <c r="I113">
+        <v>7638</v>
+      </c>
+    </row>
+    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A114" s="3">
         <v>44927</v>
       </c>
@@ -7014,8 +7801,17 @@
       <c r="F114">
         <v>132.70500000000001</v>
       </c>
-    </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G114">
+        <v>357970</v>
+      </c>
+      <c r="H114">
+        <v>95915</v>
+      </c>
+      <c r="I114">
+        <v>8017</v>
+      </c>
+    </row>
+    <row r="115" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A115" s="3">
         <v>45017</v>
       </c>
@@ -7034,8 +7830,17 @@
       <c r="F115">
         <v>131.89099999999999</v>
       </c>
-    </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G115">
+        <v>444018</v>
+      </c>
+      <c r="H115">
+        <v>97797</v>
+      </c>
+      <c r="I115">
+        <v>8223</v>
+      </c>
+    </row>
+    <row r="116" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A116" s="3">
         <v>45108</v>
       </c>
@@ -7054,8 +7859,17 @@
       <c r="F116">
         <v>134.435</v>
       </c>
-    </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G116">
+        <v>392981</v>
+      </c>
+      <c r="H116">
+        <v>90641</v>
+      </c>
+      <c r="I116">
+        <v>7833</v>
+      </c>
+    </row>
+    <row r="117" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A117" s="3">
         <v>45200</v>
       </c>
@@ -7074,8 +7888,17 @@
       <c r="F117">
         <v>133.96299999999999</v>
       </c>
-    </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G117">
+        <v>389203</v>
+      </c>
+      <c r="H117">
+        <v>93520</v>
+      </c>
+      <c r="I117">
+        <v>7914</v>
+      </c>
+    </row>
+    <row r="118" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A118" s="3">
         <v>45292</v>
       </c>
@@ -7094,8 +7917,17 @@
       <c r="F118">
         <v>135.15799999999999</v>
       </c>
-    </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G118">
+        <v>342029</v>
+      </c>
+      <c r="H118">
+        <v>93972</v>
+      </c>
+      <c r="I118">
+        <v>7923</v>
+      </c>
+    </row>
+    <row r="119" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A119" s="3">
         <v>45383</v>
       </c>
@@ -7114,8 +7946,17 @@
       <c r="F119">
         <v>137.20699999999999</v>
       </c>
-    </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G119">
+        <v>379859</v>
+      </c>
+      <c r="H119">
+        <v>92035</v>
+      </c>
+      <c r="I119">
+        <v>7699</v>
+      </c>
+    </row>
+    <row r="120" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A120" s="3">
         <v>45474</v>
       </c>
@@ -7134,8 +7975,17 @@
       <c r="F120">
         <v>137.262</v>
       </c>
-    </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G120">
+        <v>392768</v>
+      </c>
+      <c r="H120">
+        <v>91746</v>
+      </c>
+      <c r="I120">
+        <v>7682</v>
+      </c>
+    </row>
+    <row r="121" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A121" s="3">
         <v>45566</v>
       </c>
@@ -7154,8 +8004,17 @@
       <c r="F121">
         <v>139.13300000000001</v>
       </c>
-    </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G121">
+        <v>413779</v>
+      </c>
+      <c r="H121">
+        <v>90561</v>
+      </c>
+      <c r="I121">
+        <v>7702</v>
+      </c>
+    </row>
+    <row r="122" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A122" s="3">
         <v>45658</v>
       </c>
@@ -7174,8 +8033,17 @@
       <c r="F122">
         <v>140.16499999999999</v>
       </c>
-    </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G122">
+        <v>371463</v>
+      </c>
+      <c r="H122">
+        <v>95113</v>
+      </c>
+      <c r="I122">
+        <v>7990</v>
+      </c>
+    </row>
+    <row r="123" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A123" s="3">
         <v>45748</v>
       </c>
@@ -7194,8 +8062,17 @@
       <c r="F123">
         <v>141.363</v>
       </c>
-    </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G123">
+        <v>409698</v>
+      </c>
+      <c r="H123">
+        <v>94930</v>
+      </c>
+      <c r="I123">
+        <v>8011</v>
+      </c>
+    </row>
+    <row r="124" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A124" s="3">
         <v>45839</v>
       </c>
@@ -7214,8 +8091,17 @@
       <c r="F124">
         <v>142.68799999999999</v>
       </c>
-    </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G124">
+        <v>420505</v>
+      </c>
+      <c r="H124">
+        <v>91117</v>
+      </c>
+      <c r="I124">
+        <v>7879</v>
+      </c>
+    </row>
+    <row r="125" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A125" s="3">
         <v>45931</v>
       </c>
@@ -7267,28 +8153,28 @@
         <v>8</v>
       </c>
       <c r="J1" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="O1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="P1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="Q1" s="5" t="s">
         <v>16</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="O1" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="P1" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="Q1" s="5" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
ukończono prace nad punktem 4
</commit_message>
<xml_diff>
--- a/data/dane.xlsx
+++ b/data/dane.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Przemek\Documents\moje dokumenty\studia II\praca magisterska\praca-magisterska\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CDA09B7-4C93-4FCD-99DD-552E9EF9FBE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22379E3D-A3C2-4BCE-AFC5-02ECBEE7A69C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{F84DB0BC-A1A6-46E1-A833-3076C380746F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{F84DB0BC-A1A6-46E1-A833-3076C380746F}"/>
   </bookViews>
   <sheets>
     <sheet name="miesięczne" sheetId="1" r:id="rId1"/>
@@ -490,6 +490,7 @@
             <charset val="238"/>
           </rPr>
           <t xml:space="preserve">
+linie kolejowe eksploatowane [km]
 Żródło: GUS</t>
         </r>
       </text>
@@ -568,6 +569,7 @@
             <charset val="238"/>
           </rPr>
           <t xml:space="preserve">
+linie kolejowe normalnotorowe dwu- i więcej torowe [km]
 Żródło: GUS</t>
         </r>
       </text>
@@ -594,6 +596,7 @@
             <charset val="238"/>
           </rPr>
           <t xml:space="preserve">
+drogi ekspresowe [km]
 Żródło: GUS</t>
         </r>
       </text>
@@ -620,6 +623,7 @@
             <charset val="238"/>
           </rPr>
           <t xml:space="preserve">
+autostrady [km]
 Żródło: GUS</t>
         </r>
       </text>
@@ -698,6 +702,7 @@
             <charset val="238"/>
           </rPr>
           <t xml:space="preserve">
+drogi publiczne bez autostrad [km]
 Źródło: GUS</t>
         </r>
       </text>
@@ -724,6 +729,7 @@
             <charset val="238"/>
           </rPr>
           <t xml:space="preserve">
+wydatki inwestycyjne na infrastrukturę kolejową w cenach stałych [euro]
 Źródło: OECD</t>
         </r>
       </text>
@@ -750,6 +756,7 @@
             <charset val="238"/>
           </rPr>
           <t xml:space="preserve">
+wydatki inwestycyjne na infrastrukturę drogową w cenach stałych [euro]
 Źródło: OECD</t>
         </r>
       </text>
@@ -776,6 +783,7 @@
             <charset val="238"/>
           </rPr>
           <t xml:space="preserve">
+wydatki na utrzymanie infrastruktury drogowej w cenach stałych [euro]
 Źródło: OECD</t>
         </r>
       </text>
@@ -802,6 +810,7 @@
             <charset val="238"/>
           </rPr>
           <t xml:space="preserve">
+wydatki na utrzymanie infrastruktury kolejowej w cenach stałych [euro]
 Źródło: OECD</t>
         </r>
       </text>
@@ -828,6 +837,7 @@
             <charset val="238"/>
           </rPr>
           <t xml:space="preserve">
+emisja gazów cieplarnanych w transporcie ogółem [tys. ton ekwiwalentu CO2]
 Źródło: OECD</t>
         </r>
       </text>
@@ -854,6 +864,7 @@
             <charset val="238"/>
           </rPr>
           <t xml:space="preserve">
+emisja gazów cieplarnianych w transporcie drogowym [tys. ton ekwiwalentu CO2]
 Źródło: OECD</t>
         </r>
       </text>
@@ -880,6 +891,7 @@
             <charset val="238"/>
           </rPr>
           <t xml:space="preserve">
+emisja gazów cieplarnianych w transporcie kolejowym [tys. ton ekwiwalentu CO2]
 Źródło: OECD</t>
         </r>
       </text>
@@ -894,52 +906,16 @@
     <t>data</t>
   </si>
   <si>
-    <t>linie kolejowe eksploatowane [km]</t>
-  </si>
-  <si>
     <t>linie kolejowe normalnotorowe ogółem [km]</t>
   </si>
   <si>
     <t>linie kolejowe normalnotorowe zelektryfikowane [km]</t>
   </si>
   <si>
-    <t>linie kolejowe normalnotorowe dwu- i więcej torowe [km]</t>
-  </si>
-  <si>
-    <t>drogi ekspresowe [km]</t>
-  </si>
-  <si>
-    <t>autostrady [km]</t>
-  </si>
-  <si>
     <t>lokomotywy spalinowe [szt.]</t>
   </si>
   <si>
     <t>lokomotywy elektryczne [szt.]</t>
-  </si>
-  <si>
-    <t>drogi publiczne bez autostrad [km]</t>
-  </si>
-  <si>
-    <t>wydatki inwestycyjne na infrastrukturę kolejową w cenach stałych [euro]</t>
-  </si>
-  <si>
-    <t>wydatki inwestycyjne na infrastrukturę drogową w cenach stałych [euro]</t>
-  </si>
-  <si>
-    <t>wydatki na utrzymanie infrastruktury drogowej w cenach stałych [euro]</t>
-  </si>
-  <si>
-    <t>wydatki na utrzymanie infrastruktury kolejowej w cenach stałych [euro]</t>
-  </si>
-  <si>
-    <t>emisja gazów cieplarnanych w transporcie ogółem [tys. ton ekwiwalentu CO2]</t>
-  </si>
-  <si>
-    <t>emisja gazów cieplarnianych w transporcie drogowym [tys. ton ekwiwalentu CO2]</t>
-  </si>
-  <si>
-    <t>emisja gazów cieplarnianych w transporcie kolejowym [tys. ton ekwiwalentu CO2]</t>
   </si>
   <si>
     <t>tk_pas_liczba</t>
@@ -982,6 +958,42 @@
   </si>
   <si>
     <t>td_poj_ait</t>
+  </si>
+  <si>
+    <t>ink_lin_eksp</t>
+  </si>
+  <si>
+    <t>ink_lin_dwu_el</t>
+  </si>
+  <si>
+    <t>ind_drog_ekspr</t>
+  </si>
+  <si>
+    <t>ind_autostrady</t>
+  </si>
+  <si>
+    <t>ind_pub_bez_aut</t>
+  </si>
+  <si>
+    <t>ink_wyd_inw</t>
+  </si>
+  <si>
+    <t>ind_wyd_inw</t>
+  </si>
+  <si>
+    <t>ind_wyd_ut</t>
+  </si>
+  <si>
+    <t>ink_wyd_ut</t>
+  </si>
+  <si>
+    <t>env_emis_og</t>
+  </si>
+  <si>
+    <t>env_emis_td</t>
+  </si>
+  <si>
+    <t>env_emis_tk</t>
   </si>
 </sst>
 </file>
@@ -1412,22 +1424,22 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="C1" t="s">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="D1" t="s">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="E1" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="F1" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="G1" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -5314,28 +5326,28 @@
         <v>0</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -8124,57 +8136,57 @@
     <col min="2" max="17" width="17.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="90" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" ht="60" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>8</v>
-      </c>
       <c r="J1" s="5" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="Q1" s="5" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">

</xml_diff>